<commit_message>
tune easy damage and hull absorption
</commit_message>
<xml_diff>
--- a/Data Sheets/General.xlsx
+++ b/Data Sheets/General.xlsx
@@ -183,7 +183,7 @@
     <t>Hull Damage Absorption</t>
   </si>
   <si>
-    <t>0.5</t>
+    <t>0,9</t>
   </si>
   <si>
     <t>Hull Damage Scale</t>
@@ -294,7 +294,7 @@
     <t>Multiplier</t>
   </si>
   <si>
-    <t>0.03</t>
+    <t>0,01</t>
   </si>
   <si>
     <t>0.6</t>

</xml_diff>

<commit_message>
tune hull damage test values
</commit_message>
<xml_diff>
--- a/Data Sheets/General.xlsx
+++ b/Data Sheets/General.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>/Discipline</t>
   </si>
@@ -183,19 +183,10 @@
     <t>Hull Damage Absorption</t>
   </si>
   <si>
-    <t>0,9</t>
-  </si>
-  <si>
     <t>Hull Damage Scale</t>
   </si>
   <si>
-    <t>0.01</t>
-  </si>
-  <si>
     <t>Hull Damage Scale (Without Damage Control)</t>
-  </si>
-  <si>
-    <t>0.1</t>
   </si>
   <si>
     <t>Hull Flooding Scale</t>
@@ -1287,29 +1278,29 @@
       <c r="A57" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="3" t="s">
-        <v>56</v>
+      <c r="B57" s="3">
+        <v>0.999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
+      </c>
+      <c r="B58" s="3">
+        <v>0.0001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="B59" s="3">
+        <v>0.001</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B60" s="3">
         <v>40000</v>
@@ -1317,7 +1308,7 @@
     </row>
     <row r="61">
       <c r="A61" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B61" s="3">
         <v>3</v>
@@ -1325,7 +1316,7 @@
     </row>
     <row r="62">
       <c r="A62" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B62" s="3">
         <v>50</v>
@@ -1333,7 +1324,7 @@
     </row>
     <row r="63">
       <c r="A63" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B63" s="3">
         <v>0.01</v>
@@ -1341,7 +1332,7 @@
     </row>
     <row r="64">
       <c r="A64" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B64" s="3">
         <v>0.3</v>
@@ -1349,7 +1340,7 @@
     </row>
     <row r="65">
       <c r="A65" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B65" s="3">
         <v>1</v>
@@ -1357,7 +1348,7 @@
     </row>
     <row r="67" ht="20.1" customHeight="1" s="3" customFormat="1">
       <c r="A67" s="5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>29</v>
@@ -1365,7 +1356,7 @@
     </row>
     <row r="68" ht="15" customHeight="1" s="3" customFormat="1">
       <c r="A68" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B68" s="3">
         <v>100</v>
@@ -1373,7 +1364,7 @@
     </row>
     <row r="69">
       <c r="A69" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B69" s="3">
         <v>2500</v>
@@ -1381,7 +1372,7 @@
     </row>
     <row r="70">
       <c r="A70" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B70" s="3">
         <v>10000</v>
@@ -1389,7 +1380,7 @@
     </row>
     <row r="71">
       <c r="A71" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B71" s="3">
         <v>100</v>
@@ -1397,7 +1388,7 @@
     </row>
     <row r="72">
       <c r="A72" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B72" s="3">
         <v>0.05</v>
@@ -1405,7 +1396,7 @@
     </row>
     <row r="73">
       <c r="A73" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B73" s="3">
         <v>300</v>
@@ -1413,7 +1404,7 @@
     </row>
     <row r="74">
       <c r="A74" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B74" s="3">
         <v>0.15</v>
@@ -1421,7 +1412,7 @@
     </row>
     <row r="75">
       <c r="A75" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B75" s="3">
         <v>300</v>
@@ -1429,7 +1420,7 @@
     </row>
     <row r="76">
       <c r="A76" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B76" s="3">
         <v>0.15</v>
@@ -1437,7 +1428,7 @@
     </row>
     <row r="77">
       <c r="A77" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B77" s="3">
         <v>300</v>
@@ -1445,7 +1436,7 @@
     </row>
     <row r="78">
       <c r="A78" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B78" s="3">
         <v>0.15</v>
@@ -1453,7 +1444,7 @@
     </row>
     <row r="80" ht="20.1" customHeight="1" s="3" customFormat="1">
       <c r="A80" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>29</v>
@@ -1461,7 +1452,7 @@
     </row>
     <row r="81" ht="15" customHeight="1" s="3" customFormat="1">
       <c r="A81" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B81" s="3">
         <v>6E-06</v>
@@ -1469,21 +1460,21 @@
     </row>
     <row r="84" ht="20.1" customHeight="1" s="3" customFormat="1">
       <c r="A84" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="3" customFormat="1">
       <c r="A85" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B85" s="3">
         <v>1</v>
@@ -1497,7 +1488,7 @@
     </row>
     <row r="86">
       <c r="A86" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B86" s="3">
         <v>1.15</v>
@@ -1511,7 +1502,7 @@
     </row>
     <row r="87">
       <c r="A87" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B87" s="3">
         <v>0.8</v>
@@ -1525,7 +1516,7 @@
     </row>
     <row r="88">
       <c r="A88" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B88" s="3">
         <v>0.8</v>
@@ -1539,7 +1530,7 @@
     </row>
     <row r="89">
       <c r="A89" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B89" s="3">
         <v>0.37</v>
@@ -1553,7 +1544,7 @@
     </row>
     <row r="90">
       <c r="A90" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B90" s="3">
         <v>1.9</v>
@@ -1567,13 +1558,13 @@
     </row>
     <row r="93">
       <c r="A93" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>2</v>
@@ -1581,21 +1572,21 @@
     </row>
     <row r="94">
       <c r="A94" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="96" ht="20.1" customHeight="1" s="3" customFormat="1">
       <c r="A96" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>29</v>
@@ -1603,7 +1594,7 @@
     </row>
     <row r="97" ht="15" customHeight="1" s="3" customFormat="1">
       <c r="A97" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B97" s="7">
         <v>0</v>
@@ -1611,7 +1602,7 @@
     </row>
     <row r="98">
       <c r="A98" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B98" s="7">
         <v>0</v>
@@ -1619,7 +1610,7 @@
     </row>
     <row r="99">
       <c r="A99" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B99" s="3">
         <v>0.32</v>
@@ -1627,15 +1618,15 @@
     </row>
     <row r="100">
       <c r="A100" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B101" s="3">
         <v>0</v>
@@ -1643,7 +1634,7 @@
     </row>
     <row r="103" ht="20.1" customHeight="1" s="3" customFormat="1">
       <c r="A103" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B103" s="4" t="s">
         <v>29</v>
@@ -1651,23 +1642,23 @@
     </row>
     <row r="104" ht="15" customHeight="1" s="3" customFormat="1">
       <c r="A104" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="107">
@@ -1675,7 +1666,7 @@
     </row>
     <row r="108">
       <c r="A108" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>29</v>
@@ -1683,7 +1674,7 @@
     </row>
     <row r="109">
       <c r="A109" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
normalize rollback decimals and persist hull tuning
</commit_message>
<xml_diff>
--- a/Data Sheets/General.xlsx
+++ b/Data Sheets/General.xlsx
@@ -1,19 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\AppData\LocalLow\Deep Water Studio\UBOAT\Mods\uboat-the-arcade-mod\Data Sheets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BC0EE0-C8E9-42AC-98BE-845B96F38790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" fullCalcOnLoad="1" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Marek Bartniczak</author>
+  </authors>
+  <commentList>
+    <comment ref="A64" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Marek Bartniczak:
+Damages below this threshold will never generate hidden flaws. Player also won't be informed about possible flaws.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A65" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Marek Bartniczak:
+Damages above this threshold will have the highest chance for generating hidden flaws. This doesn't mean that they will occur in 100% cases, but that the probability doesn't increase above this threshold.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="104">
   <si>
     <t>/Discipline</t>
   </si>
@@ -283,15 +330,6 @@
   </si>
   <si>
     <t>Multiplier</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>0.6</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>/Resources</t>
@@ -339,9 +377,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -393,7 +430,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.3999755851924192"/>
+        <color theme="4" tint="0.39997558519241921"/>
       </bottom>
       <diagonal/>
     </border>
@@ -411,45 +448,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="0" applyFill="1" borderId="2" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="11" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Überschrift 3" xfId="1" builtinId="18"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Marek Bartniczak</author>
-  </authors>
-  <commentList>
-    <comment ref="A64" authorId="0" shapeId="0">
-      <text>
-        <t>Marek Bartniczak:
-Damages below this threshold will never generate hidden flaws. Player also won't be informed about possible flaws.</t>
-      </text>
-    </comment>
-    <comment ref="A65" authorId="0" shapeId="0">
-      <text>
-        <t>Marek Bartniczak:
-Damages above this threshold will have the highest chance for generating hidden flaws. This doesn't mean that they will occur in 100% cases, but that the probability doesn't increase above this threshold.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -714,26 +736,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D109"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D209"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.5703125" customWidth="1" style="3"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1" style="3"/>
-    <col min="3" max="3" width="21" customWidth="1" style="3"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1" style="3"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1" style="3"/>
+    <col min="1" max="1" width="45.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -743,723 +761,723 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="3">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3">
-        <v>0</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3">
-        <v>0</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="3">
-        <v>-0.004</v>
-      </c>
-      <c r="C6" s="3">
-        <v>-0.004</v>
-      </c>
-      <c r="D6" s="3">
-        <v>-0.004</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+      <c r="B6">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+      <c r="C6">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+      <c r="D6">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3">
-        <v>0.005</v>
-      </c>
-      <c r="C7" s="3">
-        <v>0.005</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+      <c r="B7">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C7">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="D7">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="3">
-        <v>0</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0</v>
-      </c>
-      <c r="D8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="3">
-        <v>0</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="3">
-        <v>-0.0002</v>
-      </c>
-      <c r="C10" s="3">
-        <v>-0.0002</v>
-      </c>
-      <c r="D10" s="3">
-        <v>-0.0002</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="s">
+      <c r="B10">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+      <c r="C10">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+      <c r="D10">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11">
         <v>0.2</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11">
         <v>0.2</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11">
         <v>0.2</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="3">
-        <v>0</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="s">
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="3">
-        <v>0</v>
-      </c>
-      <c r="C13" s="3">
-        <v>0</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="s">
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="3">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="s">
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="3">
-        <v>0</v>
-      </c>
-      <c r="C15" s="3">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="s">
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16">
         <v>0.2</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16">
         <v>0.2</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16">
         <v>0.2</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17">
         <v>20</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17">
         <v>20</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17">
         <v>20</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18">
         <v>600</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18">
         <v>600</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18">
         <v>600</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="3">
-        <v>0.66666</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0.66666</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0.66666</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="B19">
+        <v>0.66666000000000003</v>
+      </c>
+      <c r="C19">
+        <v>0.66666000000000003</v>
+      </c>
+      <c r="D19">
+        <v>0.66666000000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20">
         <v>7</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20">
         <v>7</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20">
         <v>7</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="3">
-        <v>0</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="s">
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="3">
-        <v>0</v>
-      </c>
-      <c r="C22" s="3">
-        <v>0</v>
-      </c>
-      <c r="D22" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="s">
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="3">
-        <v>0</v>
-      </c>
-      <c r="C23" s="3">
-        <v>0</v>
-      </c>
-      <c r="D23" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="s">
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="3">
-        <v>0.035</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0.035</v>
-      </c>
-      <c r="D24" s="3">
-        <v>0.035</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="s">
+      <c r="B24">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C24">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="D24">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="3">
-        <v>0</v>
-      </c>
-      <c r="C25" s="3">
-        <v>0</v>
-      </c>
-      <c r="D25" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A27" s="5" t="s">
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28">
         <v>24</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="s">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="s">
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="s">
+      <c r="B31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32">
         <v>0.01</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="3">
-        <v>0</v>
-      </c>
-      <c r="C33" s="3" t="s">
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="38" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A38" s="5" t="s">
+    <row r="38" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="42" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A42" s="5" t="s">
+    <row r="42" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A43" s="3" t="s">
+    <row r="43" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B43">
         <v>1</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44">
         <v>1</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="3" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45">
         <v>99991650</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>46</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46">
         <v>2</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="3" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="s">
+      <c r="B47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>48</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B48">
         <v>0.15</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="3" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>49</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B49">
         <v>600</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="3" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>50</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B50">
         <v>5</v>
       </c>
     </row>
-    <row r="52" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A52" s="5" t="s">
+    <row r="52" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="53" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A53" s="3" t="s">
+    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B53">
         <v>1.8E-10</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="3" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>53</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B54">
         <v>0.4</v>
       </c>
     </row>
-    <row r="56" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A56" s="5" t="s">
+    <row r="56" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="57" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A57" s="3" t="s">
+    <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="3">
+      <c r="B57">
         <v>0.999</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="3">
-        <v>0.0001</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="s">
+      <c r="B58">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="3">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="s">
+      <c r="B59">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="3">
+      <c r="B60">
         <v>40000</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="3" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="3">
+      <c r="B61">
         <v>3</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B62">
         <v>50</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="3" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>61</v>
       </c>
-      <c r="B63" s="3">
+      <c r="B63">
         <v>0.01</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="3" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="3">
+      <c r="B64">
         <v>0.3</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="3" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>63</v>
       </c>
-      <c r="B65" s="3">
+      <c r="B65">
         <v>1</v>
       </c>
     </row>
-    <row r="67" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A67" s="5" t="s">
+    <row r="67" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A68" s="3" t="s">
+    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>65</v>
       </c>
-      <c r="B68" s="3">
+      <c r="B68">
         <v>100</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>66</v>
       </c>
-      <c r="B69" s="3">
+      <c r="B69">
         <v>2500</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>67</v>
       </c>
-      <c r="B70" s="3">
+      <c r="B70">
         <v>10000</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="3" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="3">
+      <c r="B71">
         <v>100</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>69</v>
       </c>
-      <c r="B72" s="3">
+      <c r="B72">
         <v>0.05</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="3" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>70</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B73">
         <v>300</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="3" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>71</v>
       </c>
-      <c r="B74" s="3">
+      <c r="B74">
         <v>0.15</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="3" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>72</v>
       </c>
-      <c r="B75" s="3">
+      <c r="B75">
         <v>300</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="3" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>73</v>
       </c>
-      <c r="B76" s="3">
+      <c r="B76">
         <v>0.15</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="3" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>74</v>
       </c>
-      <c r="B77" s="3">
+      <c r="B77">
         <v>300</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="3" t="s">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>75</v>
       </c>
-      <c r="B78" s="3">
+      <c r="B78">
         <v>0.15</v>
       </c>
     </row>
-    <row r="80" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A80" s="5" t="s">
+    <row r="80" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B80" s="4" t="s">
+      <c r="B80" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="81" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A81" s="3" t="s">
+    <row r="81" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>77</v>
       </c>
-      <c r="B81" s="3">
-        <v>6E-06</v>
-      </c>
-    </row>
-    <row r="84" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A84" s="5" t="s">
+      <c r="B81">
+        <v>6.0000000000000002E-6</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="3" t="s">
         <v>78</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -1472,228 +1490,224 @@
         <v>80</v>
       </c>
     </row>
-    <row r="85" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A85" s="3" t="s">
+    <row r="85" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>81</v>
       </c>
-      <c r="B85" s="3">
+      <c r="B85">
         <v>1</v>
       </c>
-      <c r="C85" s="3">
+      <c r="C85">
         <v>1.05</v>
       </c>
-      <c r="D85" s="3">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="3" t="s">
+      <c r="D85">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>82</v>
       </c>
-      <c r="B86" s="3">
-        <v>1.15</v>
-      </c>
-      <c r="C86" s="3">
+      <c r="B86">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="C86">
         <v>1.35</v>
       </c>
-      <c r="D86" s="3">
+      <c r="D86">
         <v>1.7</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="3" t="s">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>83</v>
       </c>
-      <c r="B87" s="3">
+      <c r="B87">
         <v>0.8</v>
       </c>
-      <c r="C87" s="3">
+      <c r="C87">
         <v>0.9</v>
       </c>
-      <c r="D87" s="3">
+      <c r="D87">
         <v>1</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="3" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>84</v>
       </c>
-      <c r="B88" s="3">
+      <c r="B88">
         <v>0.8</v>
       </c>
-      <c r="C88" s="3">
+      <c r="C88">
         <v>0.9</v>
       </c>
-      <c r="D88" s="3">
+      <c r="D88">
         <v>1</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="3" t="s">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>85</v>
       </c>
-      <c r="B89" s="3">
+      <c r="B89">
         <v>0.37</v>
       </c>
-      <c r="C89" s="3">
+      <c r="C89">
         <v>0.6</v>
       </c>
-      <c r="D89" s="3">
+      <c r="D89">
         <v>1</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="3" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>86</v>
       </c>
-      <c r="B90" s="3">
+      <c r="B90">
         <v>1.9</v>
       </c>
-      <c r="C90" s="3">
+      <c r="C90">
         <v>1.32</v>
       </c>
-      <c r="D90" s="3">
+      <c r="D90">
         <v>0.9</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="3" t="s">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>87</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="B93" t="s">
         <v>79</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" t="s">
         <v>88</v>
       </c>
-      <c r="D93" s="3" t="s">
+      <c r="D93" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="3" t="s">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>89</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="B94" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="C94">
+        <v>0.6</v>
+      </c>
+      <c r="D94" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C94" s="3" t="s">
+      <c r="B96" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>91</v>
       </c>
-      <c r="D94" s="3" t="s">
+      <c r="B97" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="96" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A96" s="5" t="s">
+      <c r="B98" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>93</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B99">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>94</v>
+      </c>
+      <c r="B100" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>96</v>
+      </c>
+      <c r="B101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B103" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="97" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A97" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B97" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B98" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B99" s="3">
-        <v>0.32</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B100" s="3" t="s">
+    <row r="104" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="3" t="s">
+      <c r="B104" t="s">
         <v>99</v>
       </c>
-      <c r="B101" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" ht="20.1" customHeight="1" s="3" customFormat="1">
-      <c r="A103" s="5" t="s">
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>100</v>
       </c>
-      <c r="B103" s="4" t="s">
+      <c r="B105" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>102</v>
+      </c>
+      <c r="B108" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="104" ht="15" customHeight="1" s="3" customFormat="1">
-      <c r="A104" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="3" t="s">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>103</v>
       </c>
-      <c r="B105" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="3"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B108" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B109" s="3" t="s">
+      <c r="B109" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="112" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="121" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="129" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="137" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="143" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="147" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="157" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="165" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="189" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="208" ht="15" customHeight="1" s="3" customFormat="1"/>
-    <row r="209" ht="15" customHeight="1" s="3" customFormat="1"/>
+    <row r="112" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="121" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="129" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="137" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="143" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="157" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="209" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
rollback hull damage factors to vanilla
</commit_message>
<xml_diff>
--- a/Data Sheets/General.xlsx
+++ b/Data Sheets/General.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0" iterateDelta="1E-4" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>/Discipline</t>
   </si>
@@ -378,7 +378,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,14 +449,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="0" applyFill="1" borderId="2" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="3" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="11" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -737,21 +739,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D209"/>
+  <dimension ref="A1:D109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1"/>
+    <col min="1" max="1" width="45.5703125" customWidth="1" style="2"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1" style="2"/>
+    <col min="3" max="3" width="21" customWidth="1" style="2"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1" style="2"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" ht="20.1" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -761,723 +763,723 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B3" s="2">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
-        <v>-4.0000000000000001E-3</v>
-      </c>
-      <c r="C6">
-        <v>-4.0000000000000001E-3</v>
-      </c>
-      <c r="D6">
-        <v>-4.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B6" s="2">
+        <v>-0.004</v>
+      </c>
+      <c r="C6" s="2">
+        <v>-0.004</v>
+      </c>
+      <c r="D6" s="2">
+        <v>-0.004</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C7">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="D7">
-        <v>5.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B7" s="2">
+        <v>0.005</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.005</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="B9" s="2">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10">
-        <v>-2.0000000000000001E-4</v>
-      </c>
-      <c r="C10">
-        <v>-2.0000000000000001E-4</v>
-      </c>
-      <c r="D10">
-        <v>-2.0000000000000001E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="B10" s="2">
+        <v>-0.0002</v>
+      </c>
+      <c r="C10" s="2">
+        <v>-0.0002</v>
+      </c>
+      <c r="D10" s="2">
+        <v>-0.0002</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="2">
         <v>0.2</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="2">
         <v>0.2</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>0.2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12">
+      <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B13">
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="B13" s="2">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B14">
-        <v>0</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="B15" s="2">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="2">
         <v>0.2</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="2">
         <v>0.2</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    <row r="17">
+      <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="2">
         <v>20</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="2">
         <v>20</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+    <row r="18">
+      <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="2">
         <v>600</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="2">
         <v>600</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>600</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+    <row r="19">
+      <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B19">
-        <v>0.66666000000000003</v>
-      </c>
-      <c r="C19">
-        <v>0.66666000000000003</v>
-      </c>
-      <c r="D19">
-        <v>0.66666000000000003</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="B19" s="2">
+        <v>0.66666</v>
+      </c>
+      <c r="C19" s="2">
+        <v>0.66666</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.66666</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="2">
         <v>7</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="2">
         <v>7</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+    <row r="21">
+      <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="B21" s="2">
+        <v>0</v>
+      </c>
+      <c r="C21" s="2">
+        <v>0</v>
+      </c>
+      <c r="D21" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="B22" s="2">
+        <v>0</v>
+      </c>
+      <c r="C22" s="2">
+        <v>0</v>
+      </c>
+      <c r="D22" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="B23" s="2">
+        <v>0</v>
+      </c>
+      <c r="C23" s="2">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B24">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="C24">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="D24">
-        <v>3.5000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="B24" s="2">
+        <v>0.035</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.035</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B25">
-        <v>0</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+      <c r="B25" s="2">
+        <v>0</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="20.1" customHeight="1">
+      <c r="A27" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29">
+      <c r="A29" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B29" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B30" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B31" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="2">
         <v>0.01</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33">
+      <c r="A33" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B33">
-        <v>0</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B33" s="2">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34">
+      <c r="A34" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35">
+      <c r="A35" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
+    <row r="38" ht="20.1" customHeight="1">
+      <c r="A38" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
+    <row r="42" ht="20.1" customHeight="1">
+      <c r="A42" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44">
+      <c r="A44" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45">
+      <c r="A45" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="2">
         <v>99991650</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46">
+      <c r="A46" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47">
+      <c r="A47" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="B47" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49">
+      <c r="A49" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="2">
         <v>600</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50">
+      <c r="A50" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
+    <row r="52" ht="20.1" customHeight="1">
+      <c r="A52" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="2">
         <v>1.8E-10</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54">
+      <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="2">
         <v>0.4</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="3" t="s">
+    <row r="56" ht="20.1" customHeight="1">
+      <c r="A56" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B57">
-        <v>0.999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="B57" s="2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B58">
-        <v>1E-4</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="B58" s="2">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B59">
-        <v>1E-3</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="B59" s="2">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="2">
         <v>40000</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="61">
+      <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="62">
+      <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="63">
+      <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="2">
         <v>0.01</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="64">
+      <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="2">
         <v>0.3</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="65">
+      <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
+    <row r="67" ht="20.1" customHeight="1">
+      <c r="A67" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="68" ht="15" customHeight="1">
+      <c r="A68" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="69">
+      <c r="A69" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="2">
         <v>2500</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="70">
+      <c r="A70" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="2">
         <v>10000</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="71">
+      <c r="A71" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="72">
+      <c r="A72" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="2">
         <v>0.05</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="73">
+      <c r="A73" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="2">
         <v>300</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="74">
+      <c r="A74" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="75">
+      <c r="A75" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="2">
         <v>300</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="76">
+      <c r="A76" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B76">
+      <c r="B76" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="77">
+      <c r="A77" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B77">
+      <c r="B77" s="2">
         <v>300</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="78">
+      <c r="A78" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B78">
+      <c r="B78" s="2">
         <v>0.15</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="3" t="s">
+    <row r="80" ht="20.1" customHeight="1">
+      <c r="A80" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B81">
-        <v>6.0000000000000002E-6</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="3" t="s">
+      <c r="B81" s="2">
+        <v>6E-06</v>
+      </c>
+    </row>
+    <row r="84" ht="20.1" customHeight="1">
+      <c r="A84" s="4" t="s">
         <v>78</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -1490,224 +1492,225 @@
         <v>80</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B85">
+      <c r="B85" s="2">
         <v>1</v>
       </c>
-      <c r="C85">
+      <c r="C85" s="2">
         <v>1.05</v>
       </c>
-      <c r="D85">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+      <c r="D85" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B86">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C86">
+      <c r="B86" s="2">
+        <v>1.15</v>
+      </c>
+      <c r="C86" s="2">
         <v>1.35</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="2">
         <v>1.7</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="87">
+      <c r="A87" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B87">
+      <c r="B87" s="2">
         <v>0.8</v>
       </c>
-      <c r="C87">
+      <c r="C87" s="2">
         <v>0.9</v>
       </c>
-      <c r="D87">
+      <c r="D87" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="88">
+      <c r="A88" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B88">
+      <c r="B88" s="2">
         <v>0.8</v>
       </c>
-      <c r="C88">
+      <c r="C88" s="2">
         <v>0.9</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="89">
+      <c r="A89" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B89">
+      <c r="B89" s="2">
         <v>0.37</v>
       </c>
-      <c r="C89">
+      <c r="C89" s="2">
         <v>0.6</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="90">
+      <c r="A90" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B90">
+      <c r="B90" s="2">
         <v>1.9</v>
       </c>
-      <c r="C90">
+      <c r="C90" s="2">
         <v>1.32</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="2">
         <v>0.9</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="93">
+      <c r="A93" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C93" t="s">
+      <c r="C93" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D93" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="94">
+      <c r="A94" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B94" s="6">
+      <c r="B94" s="7">
         <v>0.01</v>
       </c>
-      <c r="C94">
+      <c r="C94" s="2">
         <v>0.6</v>
       </c>
-      <c r="D94" s="6">
+      <c r="D94" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="3" t="s">
+    <row r="96" ht="20.1" customHeight="1">
+      <c r="A96" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B97" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="B97" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B98" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="B98" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B99">
+      <c r="B99" s="2">
         <v>0.32</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="100">
+      <c r="A100" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="101">
+      <c r="A101" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="3" t="s">
+      <c r="B101" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" ht="20.1" customHeight="1">
+      <c r="A103" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="105">
+      <c r="A105" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+    <row r="106">
+      <c r="A106" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+    <row r="108">
+      <c r="A108" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+    <row r="109">
+      <c r="A109" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="208" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="209" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="129" ht="15" customHeight="1"/>
+    <row r="137" ht="15" customHeight="1"/>
+    <row r="143" ht="15" customHeight="1"/>
+    <row r="147" ht="15" customHeight="1"/>
+    <row r="157" ht="15" customHeight="1"/>
+    <row r="165" ht="15" customHeight="1"/>
+    <row r="189" ht="15" customHeight="1"/>
+    <row r="208" ht="15" customHeight="1"/>
+    <row r="209" ht="15" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
verify player ship damage scale and close damage todo
</commit_message>
<xml_diff>
--- a/Data Sheets/General.xlsx
+++ b/Data Sheets/General.xlsx
@@ -449,9 +449,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="1" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="1" applyBorder="1" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" applyNumberFormat="1" fontId="2" applyFont="1" fillId="0" applyFill="1" borderId="2" applyBorder="1" xfId="0" applyProtection="1"/>
@@ -742,18 +743,18 @@
   <dimension ref="A1:D109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.5703125" customWidth="1" style="2"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1" style="2"/>
-    <col min="3" max="3" width="21" customWidth="1" style="2"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1" style="2"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1" style="2"/>
+    <col min="1" max="1" width="45.5703125" customWidth="1" style="3"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1" style="3"/>
+    <col min="3" max="3" width="21" customWidth="1" style="3"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1" style="3"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.1" customHeight="1">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -764,722 +765,722 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="B2" s="3">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="B4" s="3">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>-0.004</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>-0.004</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>-0.004</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>0.005</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>0.005</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>0.005</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="B8" s="3">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2">
-        <v>0</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="B9" s="3">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>-0.0002</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>-0.0002</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="3">
         <v>-0.0002</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="3">
         <v>0.2</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>0.2</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="3">
         <v>0.2</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="2">
-        <v>0</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2">
+      <c r="B12" s="3">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="2">
-        <v>0</v>
-      </c>
-      <c r="C13" s="2">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2">
+      <c r="B13" s="3">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="2">
-        <v>0</v>
-      </c>
-      <c r="C14" s="2">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2">
+      <c r="B14" s="3">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="2">
-        <v>0</v>
-      </c>
-      <c r="C15" s="2">
-        <v>0</v>
-      </c>
-      <c r="D15" s="2">
+      <c r="B15" s="3">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="3">
         <v>0.2</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>0.2</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="3">
         <v>0.2</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="3">
         <v>20</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <v>20</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="3">
         <v>20</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="3">
         <v>600</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>600</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="3">
         <v>600</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="3">
         <v>0.66666</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <v>0.66666</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="3">
         <v>0.66666</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="3">
         <v>7</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="3">
         <v>7</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="3">
         <v>7</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="2">
-        <v>0</v>
-      </c>
-      <c r="C21" s="2">
-        <v>0</v>
-      </c>
-      <c r="D21" s="2">
+      <c r="B21" s="3">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="2">
-        <v>0</v>
-      </c>
-      <c r="C22" s="2">
-        <v>0</v>
-      </c>
-      <c r="D22" s="2">
+      <c r="B22" s="3">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="2">
-        <v>0</v>
-      </c>
-      <c r="C23" s="2">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2">
+      <c r="B23" s="3">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="3">
         <v>0.035</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="3">
         <v>0.035</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="3">
         <v>0.035</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="2">
-        <v>0</v>
-      </c>
-      <c r="C25" s="2">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2">
+      <c r="B25" s="3">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="27" ht="20.1" customHeight="1">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="3">
         <v>24</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="3">
         <v>0.01</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="2">
-        <v>0</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="B33" s="3">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="38" ht="20.1" customHeight="1">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="42" ht="20.1" customHeight="1">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="3">
         <v>99991650</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="3">
         <v>2</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="3">
         <v>0.15</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="3">
         <v>600</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="s">
+      <c r="A50" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="52" ht="20.1" customHeight="1">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="2" t="s">
+      <c r="A53" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="3">
         <v>1.8E-10</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="s">
+      <c r="A54" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="3">
         <v>0.4</v>
       </c>
     </row>
     <row r="56" ht="20.1" customHeight="1">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="B56" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="2" t="s">
+      <c r="A57" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="3">
         <v>0.2</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="3">
         <v>0.43</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="s">
+      <c r="A59" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="3">
         <v>0.86</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="3">
         <v>40000</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="2">
-        <v>3</v>
+      <c r="B61" s="3">
+        <v>0.1</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="3">
         <v>50</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="s">
+      <c r="A63" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="3">
         <v>0.01</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="s">
+      <c r="A64" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="3">
         <v>0.3</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="67" ht="20.1" customHeight="1">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B67" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="2" t="s">
+      <c r="A68" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="3">
         <v>100</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="s">
+      <c r="A69" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="3">
         <v>2500</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="s">
+      <c r="A70" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="3">
         <v>10000</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="s">
+      <c r="A71" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="3">
         <v>100</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="s">
+      <c r="A72" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="3">
         <v>0.05</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="s">
+      <c r="A73" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="3">
         <v>300</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="s">
+      <c r="A74" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B74" s="2">
+      <c r="B74" s="3">
         <v>0.15</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="s">
+      <c r="A75" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B75" s="2">
+      <c r="B75" s="3">
         <v>300</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="s">
+      <c r="A76" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B76" s="3">
         <v>0.15</v>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="s">
+      <c r="A77" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B77" s="3">
         <v>300</v>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="s">
+      <c r="A78" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B78" s="3">
         <v>0.15</v>
       </c>
     </row>
     <row r="80" ht="20.1" customHeight="1">
-      <c r="A80" s="4" t="s">
+      <c r="A80" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="2" t="s">
+      <c r="A81" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B81" s="2">
+      <c r="B81" s="3">
         <v>6E-06</v>
       </c>
     </row>
     <row r="84" ht="20.1" customHeight="1">
-      <c r="A84" s="4" t="s">
+      <c r="A84" s="5" t="s">
         <v>78</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -1493,207 +1494,207 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="2" t="s">
+      <c r="A85" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B85" s="2">
+      <c r="B85" s="3">
         <v>1</v>
       </c>
-      <c r="C85" s="2">
+      <c r="C85" s="3">
         <v>1.05</v>
       </c>
-      <c r="D85" s="2">
+      <c r="D85" s="3">
         <v>1.1</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="s">
+      <c r="A86" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B86" s="2">
+      <c r="B86" s="3">
         <v>1.15</v>
       </c>
-      <c r="C86" s="2">
+      <c r="C86" s="3">
         <v>1.35</v>
       </c>
-      <c r="D86" s="2">
+      <c r="D86" s="3">
         <v>1.7</v>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="s">
+      <c r="A87" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B87" s="2">
+      <c r="B87" s="3">
         <v>0.8</v>
       </c>
-      <c r="C87" s="2">
+      <c r="C87" s="3">
         <v>0.9</v>
       </c>
-      <c r="D87" s="2">
+      <c r="D87" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="s">
+      <c r="A88" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B88" s="2">
+      <c r="B88" s="3">
         <v>0.8</v>
       </c>
-      <c r="C88" s="2">
+      <c r="C88" s="3">
         <v>0.9</v>
       </c>
-      <c r="D88" s="2">
+      <c r="D88" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="s">
+      <c r="A89" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B89" s="2">
+      <c r="B89" s="3">
         <v>0.37</v>
       </c>
-      <c r="C89" s="2">
+      <c r="C89" s="3">
         <v>0.6</v>
       </c>
-      <c r="D89" s="2">
+      <c r="D89" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="s">
+      <c r="A90" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B90" s="2">
+      <c r="B90" s="3">
         <v>1.9</v>
       </c>
-      <c r="C90" s="2">
+      <c r="C90" s="3">
         <v>1.32</v>
       </c>
-      <c r="D90" s="2">
+      <c r="D90" s="3">
         <v>0.9</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="s">
+      <c r="A93" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B93" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C93" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D93" s="2" t="s">
+      <c r="D93" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="s">
+      <c r="A94" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B94" s="7">
+      <c r="B94" s="8">
         <v>0.01</v>
       </c>
-      <c r="C94" s="2">
+      <c r="C94" s="3">
         <v>0.6</v>
       </c>
-      <c r="D94" s="7">
+      <c r="D94" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="96" ht="20.1" customHeight="1">
-      <c r="A96" s="4" t="s">
+      <c r="A96" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="B96" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="2" t="s">
+      <c r="A97" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B97" s="6">
+      <c r="B97" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="s">
+      <c r="A98" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B98" s="6">
+      <c r="B98" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B99" s="2">
+      <c r="B99" s="3">
         <v>0.32</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="s">
+      <c r="A100" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" s="3" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="s">
+      <c r="A101" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B101" s="2">
+      <c r="B101" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="103" ht="20.1" customHeight="1">
-      <c r="A103" s="4" t="s">
+      <c r="A103" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B103" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="2" t="s">
+      <c r="A104" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B104" s="3" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="s">
+      <c r="A105" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B105" s="2" t="s">
+      <c r="B105" s="3" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="s">
+      <c r="A106" s="3" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="s">
+      <c r="A108" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B108" s="2" t="s">
+      <c r="B108" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="s">
+      <c r="A109" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="B109" s="3" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>